<commit_message>
fix: "nationality": "male" updated to "nationality": "albania"
</commit_message>
<xml_diff>
--- a/input/_metadata.xlsx
+++ b/input/_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tolgahanturker/Desktop/auto-filler/taxonomy-auto-filler/res/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tolgahanturker/Desktop/auto-extender/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA31517-0388-D74A-BAB6-DC56543490C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E4461E-4379-DF4A-B18A-A56FC2452C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35840" windowHeight="20060" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mini-corpus-147" sheetId="1" r:id="rId1"/>
@@ -618,6 +618,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -625,16 +626,19 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -645,12 +649,14 @@
       <sz val="10"/>
       <color rgb="FFFF9900"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -16570,7 +16576,7 @@
         <v>255</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="C141" s="5" t="s">
         <v>9</v>

</xml_diff>